<commit_message>
UI: Reorder QR payment section and remove duplicate Pay Now button
</commit_message>
<xml_diff>
--- a/exports/donations.xlsx
+++ b/exports/donations.xlsx
@@ -419,7 +419,7 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="5" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -504,17 +504,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DON-3E6C0534</t>
+          <t>DON-C16DAB40</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>121212</t>
+          <t>111111</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ravi</t>
+          <t>Kona Meghana</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -522,7 +522,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>tirupathi</t>
+          <t>Anantapur</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2700</v>
+        <v>2500</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -545,7 +545,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>donation_1779095630_hero.png.png</t>
+          <t>donation_1779090841_hero.png.png</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">

</xml_diff>